<commit_message>
feat(IEEE14): Resolving TCSC problems due to issues in modeling
</commit_message>
<xml_diff>
--- a/01_Data/03_Test_Cases/IEEE 14/03_Escenarios/01 - wo Stress/caso_IEEE14_E2_24h.xlsx
+++ b/01_Data/03_Test_Cases/IEEE 14/03_Escenarios/01 - wo Stress/caso_IEEE14_E2_24h.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\2. Universidad Nacional de Colombia\2. Postgraduate\1_SEMESTER\TESIS DE MAESTRIA\2nd Search\04_TESIS_DANIEL\03_CODIGO_TRABAJO_DANIEL\BESS_FACTS_master\01_Data\03_Test_Cases\IEEE 14\03_Escenarios\01 - wo Stress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17BE934E-4386-4775-BDEE-661C56D80865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB5E6F98-24BF-4322-B233-EFE42B3C09BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCCIONES" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="161">
   <si>
     <t>Plantilla de datos - Modelo TEP con BESS y FACTS</t>
   </si>
@@ -386,12 +386,6 @@
     <t>linea</t>
   </si>
   <si>
-    <t>dB_min</t>
-  </si>
-  <si>
-    <t>dB_max</t>
-  </si>
-  <si>
     <t>Demanda - Perfil horario de demanda por nodo</t>
   </si>
   <si>
@@ -552,6 +546,24 @@
   </si>
   <si>
     <t>CREG</t>
+  </si>
+  <si>
+    <t>habilitada</t>
+  </si>
+  <si>
+    <t>sigma_niveles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	-0.20,-0.10,0.15,0.30,0.45,0.60</t>
+  </si>
+  <si>
+    <t>[USD/MVAr]</t>
+  </si>
+  <si>
+    <t>c_tcsc</t>
+  </si>
+  <si>
+    <t>theta_max_grados</t>
   </si>
 </sst>
 </file>
@@ -562,7 +574,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -617,13 +629,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -667,10 +672,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -709,16 +713,15 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="6" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Comma" xfId="2" builtinId="3"/>
+  <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -1141,7 +1144,7 @@
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
@@ -1154,7 +1157,7 @@
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
@@ -1167,326 +1170,192 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="16" customWidth="1"/>
+    <col min="1" max="2" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>100</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
-      <c r="B5" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="4"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B6" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C6" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D6" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="B8" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C7" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D7" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="B9" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B8" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C8" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D8" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+      <c r="B10" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B9" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C9" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D9" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="B11" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B10" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C10" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D10" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="B12" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B11" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C11" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D11" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="B13" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B12" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C12" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D12" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="B14" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C13" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D13" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="B15" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B14" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C14" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D14" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="B15" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C15" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D15" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>124</v>
-      </c>
       <c r="B16" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C16" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D16" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="B17" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B18" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="B17" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C17" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D17" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
+      <c r="B19" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="B18" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C18" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D18" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="B20" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="B19" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C19" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D19" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="B21" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B20" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C20" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D20" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+      <c r="B22" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B21" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C21" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D21" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
+      <c r="B23" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="B22" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C22" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D22" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+      <c r="B24" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="B23" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C23" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D23" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="B24" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C24" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D24" s="14">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
-        <v>150</v>
-      </c>
       <c r="B25" s="5">
-        <v>-0.7</v>
-      </c>
-      <c r="C25" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D25" s="14">
-        <v>50000</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1504,23 +1373,23 @@
   <sheetData>
     <row r="1" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>41</v>
@@ -1532,22 +1401,22 @@
         <v>43</v>
       </c>
       <c r="G4" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>139</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -2506,11 +2375,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
     <col min="3" max="3" width="35.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2608,46 +2477,73 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B12" s="7">
         <v>15</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B13" s="7">
         <v>20</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B14" s="11">
         <v>1</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B15" s="11">
         <v>0.115</v>
       </c>
       <c r="C15" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="B16" s="11">
+        <v>135000</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="16" t="s">
         <v>156</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="B18" s="11">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -2696,10 +2592,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C6" s="5">
         <v>0</v>
@@ -2707,10 +2603,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C7" s="5">
         <v>21.7</v>
@@ -2718,10 +2614,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C8" s="5">
         <v>94.2</v>
@@ -2732,7 +2628,7 @@
         <v>41</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C9" s="5">
         <v>47.8</v>
@@ -2743,7 +2639,7 @@
         <v>42</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C10" s="5">
         <v>7.6</v>
@@ -2754,7 +2650,7 @@
         <v>43</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C11" s="5">
         <v>11.2</v>
@@ -2762,10 +2658,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C12" s="5">
         <v>0</v>
@@ -2773,10 +2669,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C13" s="5">
         <v>0</v>
@@ -2784,10 +2680,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C14" s="5">
         <v>29.5</v>
@@ -2795,10 +2691,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C15" s="5">
         <v>9</v>
@@ -2806,10 +2702,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C16" s="5">
         <v>3.5</v>
@@ -2817,10 +2713,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C17" s="5">
         <v>6.1</v>
@@ -2828,10 +2724,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C18" s="5">
         <v>13.5</v>
@@ -2839,10 +2735,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C19" s="5">
         <v>14.9</v>
@@ -2912,13 +2808,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D6" s="5">
         <v>1.9380000000000001E-2</v>
@@ -2926,16 +2822,16 @@
       <c r="E6" s="5">
         <v>5.917E-2</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="15">
         <v>155.60399999999998</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>42</v>
@@ -2946,19 +2842,19 @@
       <c r="E7" s="5">
         <v>0.22303999999999999</v>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="15">
         <v>77.591999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D8" s="5">
         <v>4.6989999999999997E-2</v>
@@ -2966,16 +2862,16 @@
       <c r="E8" s="5">
         <v>0.19797000000000001</v>
       </c>
-      <c r="F8" s="16">
+      <c r="F8" s="15">
         <v>66.707999999999998</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>41</v>
@@ -2986,16 +2882,16 @@
       <c r="E9" s="5">
         <v>0.17632</v>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="15">
         <v>58.704000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>42</v>
@@ -3006,16 +2902,16 @@
       <c r="E10" s="5">
         <v>0.17388000000000001</v>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="15">
         <v>44.735999999999997</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>41</v>
@@ -3026,13 +2922,13 @@
       <c r="E11" s="5">
         <v>0.17102999999999999</v>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="15">
         <v>13.452</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>41</v>
@@ -3046,19 +2942,19 @@
       <c r="E12" s="5">
         <v>4.2110000000000002E-2</v>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="15">
         <v>59.003999999999998</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>41</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D13" s="5">
         <v>0</v>
@@ -3066,19 +2962,19 @@
       <c r="E13" s="5">
         <v>0.20912</v>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="15">
         <v>27.42</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>41</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D14" s="5">
         <v>0</v>
@@ -3086,13 +2982,13 @@
       <c r="E14" s="5">
         <v>0.55618000000000001</v>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="15">
         <v>17.808</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>42</v>
@@ -3106,19 +3002,19 @@
       <c r="E15" s="5">
         <v>0.25202000000000002</v>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="15">
         <v>50.472000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D16" s="5">
         <v>9.4979999999999995E-2</v>
@@ -3126,19 +3022,19 @@
       <c r="E16" s="5">
         <v>0.19889999999999999</v>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="15">
         <v>7.3079999999999998</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D17" s="5">
         <v>0.12291000000000001</v>
@@ -3146,19 +3042,19 @@
       <c r="E17" s="5">
         <v>0.25580999999999998</v>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="15">
         <v>9.18</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D18" s="5">
         <v>6.615E-2</v>
@@ -3166,19 +3062,19 @@
       <c r="E18" s="5">
         <v>0.13027</v>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="15">
         <v>20.544</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D19" s="5">
         <v>0</v>
@@ -3186,19 +3082,19 @@
       <c r="E19" s="5">
         <v>0.17615</v>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="15">
         <v>10.188000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B20" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>136</v>
       </c>
       <c r="D20" s="5">
         <v>0</v>
@@ -3206,19 +3102,19 @@
       <c r="E20" s="5">
         <v>0.11001</v>
       </c>
-      <c r="F20" s="16">
+      <c r="F20" s="15">
         <v>37.607999999999997</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D21" s="5">
         <v>3.1809999999999998E-2</v>
@@ -3226,19 +3122,19 @@
       <c r="E21" s="5">
         <v>8.4500000000000006E-2</v>
       </c>
-      <c r="F21" s="16">
+      <c r="F21" s="15">
         <v>7.7880000000000003</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D22" s="5">
         <v>0.12711</v>
@@ -3246,19 +3142,19 @@
       <c r="E22" s="5">
         <v>0.27038000000000001</v>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="15">
         <v>12.239999999999998</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D23" s="5">
         <v>8.2049999999999998E-2</v>
@@ -3266,19 +3162,19 @@
       <c r="E23" s="5">
         <v>0.19206999999999999</v>
       </c>
-      <c r="F23" s="16">
+      <c r="F23" s="15">
         <v>3.0359999999999996</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D24" s="5">
         <v>0.22092000000000001</v>
@@ -3286,19 +3182,19 @@
       <c r="E24" s="5">
         <v>0.19988</v>
       </c>
-      <c r="F24" s="16">
+      <c r="F24" s="15">
         <v>1.776</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D25" s="5">
         <v>0.17093</v>
@@ -3306,7 +3202,7 @@
       <c r="E25" s="5">
         <v>0.34802</v>
       </c>
-      <c r="F25" s="16">
+      <c r="F25" s="15">
         <v>5.8559999999999999</v>
       </c>
     </row>
@@ -3427,7 +3323,7 @@
         <v>64</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>65</v>
@@ -3479,10 +3375,10 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C6" s="5">
         <v>0</v>
@@ -3522,10 +3418,10 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C7" s="5">
         <v>0</v>
@@ -3565,10 +3461,10 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C8" s="5">
         <v>0</v>
@@ -3607,7 +3503,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>43</v>
@@ -3649,10 +3545,10 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C10" s="5">
         <v>0</v>
@@ -3892,7 +3788,7 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C7" s="15"/>
+      <c r="C7" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>